<commit_message>
Replace real organization names in seed, tests, mockups and docs with generic ones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019WHQmhFu6UJU12sLXYK4ET
</commit_message>
<xml_diff>
--- a/web/public/sample_assets_messy.xlsx
+++ b/web/public/sample_assets_messy.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>정보화담당관실</t>
+          <t>정보화팀</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>도로국</t>
+          <t>시설관리과</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>